<commit_message>
Use single excel dataset and add context memory
</commit_message>
<xml_diff>
--- a/QA_Dataset_1000_Chatbot.xlsx
+++ b/QA_Dataset_1000_Chatbot.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\doc-sheet-chatbot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D6FEBD-7EDD-4A53-82E8-A50D84A20E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD949DC9-6330-4138-A081-E4B71E99F579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QA_Dataset_1000" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1905" uniqueCount="1084">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2003" uniqueCount="1182">
   <si>
     <t>ลำดับข้อ</t>
   </si>
@@ -3428,6 +3441,309 @@
   </si>
   <si>
     <t>สรุปวิธีและแนวทางปฏิบัติของ การจัดทำแผนการจัดการเรียนรู้ของครูอาชีวศึกษา สอดคล้องและสัมพันธ์กับหนังสือการออกแบบการจัดการเรียนรู้ของ ศ.ดร.ชัยวัฒน์ สุทธิรัตน์ ให้ทีครับ/ค่ะ</t>
+  </si>
+  <si>
+    <t>แผนการสอนนี้เป็นของสถาบันหรือหน่วยงานใด?</t>
+  </si>
+  <si>
+    <t>แบบฟอร์มแผนการสอน คณะครุศาสตร์อุตสาหกรรม มจพ. มีโครงสร้างส่วนหัวอย่างไร?</t>
+  </si>
+  <si>
+    <t>ข้อมูลพื้นฐานส่วนหัวของแบบฟอร์มแผนการสอน มจพ. มีอะไรบ้าง?</t>
+  </si>
+  <si>
+    <t>ในแบบฟอร์มระบุระดับชั้นเรียนและกลุ่มเรียนตัวอย่างเป็นอะไร?</t>
+  </si>
+  <si>
+    <t>เวลาในการสอนในแบบฟอร์มกำหนดหน่วยเป็นอะไร?</t>
+  </si>
+  <si>
+    <t>ส่วนหัวของแผนการสอนต้องระบุชื่อผู้สอนและปีการศึกษาหรือไม่?</t>
+  </si>
+  <si>
+    <t>วัตถุประสงค์ในแผนการสอนระบุเป็นประเภทใด?</t>
+  </si>
+  <si>
+    <t>การเขียนวัตถุประสงค์เชิงพฤติกรรมในแผนการสอนมีข้อความนำอย่างไร?</t>
+  </si>
+  <si>
+    <t>ในแบบฟอร์มให้จับคู่วัตถุประสงค์เชิงพฤติกรรมกับการประเมินส่วนใด?</t>
+  </si>
+  <si>
+    <t>การประเมินขั้นสำเร็จผลในแผนการสอนมีความสัมพันธ์กับวัตถุประสงค์อย่างไร?</t>
+  </si>
+  <si>
+    <t>วัตถุประสงค์เชิงพฤติกรรมในแบบฟอร์มเว้นไว้กี่ข้อ?</t>
+  </si>
+  <si>
+    <t>ช่อง 'ความรู้พื้นฐานที่จำเป็น' มีไว้สำหรับระบุอะไร?</t>
+  </si>
+  <si>
+    <t>ช่อง 'การนำเข้าสู่บทเรียน' มีความสำคัญอย่างไรในแผน?</t>
+  </si>
+  <si>
+    <t>ทำไมแผนการสอนต้องระบุความรู้พื้นฐานที่จำเป็นก่อนเริ่มสอน?</t>
+  </si>
+  <si>
+    <t>รูปแบบขั้นตอนการสอนหลักในตารางปฏิบัติการมีกี่ขั้นตอน อะไรบ้าง?</t>
+  </si>
+  <si>
+    <t>ขั้นบอกกล่าวใช้ตัวอักษรย่อภาษาอังกฤษว่าอะไร?</t>
+  </si>
+  <si>
+    <t>ขั้นพยายามใช้ตัวอักษรย่อภาษาอังกฤษว่าอะไร?</t>
+  </si>
+  <si>
+    <t>ขั้นสำเร็จผลใช้ตัวอักษรย่อภาษาอังกฤษว่าอะไร?</t>
+  </si>
+  <si>
+    <t>เป็นแบบฟอร์มแผนการสอนของ คณะครุศาสตร์อุตสาหกรรม มหาวิทยาลัยเทคโนโลยีพระจอมเกล้าพระนครเหนือ (มจพ.)</t>
+  </si>
+  <si>
+    <t>ระบุชื่อสถาบัน คณะครุศาสตร์อุตสาหกรรม มจพ., เรื่อง, วิชา, เวลาในการสอน (นาที), ชั้นเรียน, วันที่สอน, ผู้สอน, ชั้น/กลุ่มเรียน และปีการศึกษา</t>
+  </si>
+  <si>
+    <t>ประกอบด้วย คณะ/สถาบัน, เรื่อง, วิชา, เวลาในการสอน (นาที), ชั้นเรียน, วันที่สอน, ผู้สอน, ชั้น/กลุ่มเรียน และปีการศึกษา</t>
+  </si>
+  <si>
+    <t>ระบุระดับชั้นเรียน ปวช.1 และกลุ่มเรียน ชั้น TCT1-DERA</t>
+  </si>
+  <si>
+    <t>มีช่องระบุเวลาในการสอนเป็นหน่วย 'นาที'</t>
+  </si>
+  <si>
+    <t>ต้องระบุ โดยมีช่องสำหรับกรอกชื่อผู้สอน ชั้น/กลุ่มเรียน และปีการศึกษาอย่างชัดเจน</t>
+  </si>
+  <si>
+    <t>ระบุเป็น 'วัตถุประสงค์เชิงพฤติกรรม' (Behavioral Objectives)</t>
+  </si>
+  <si>
+    <t>มีข้อความนำระบุว่า 'หลังจบการเรียนการสอนผู้เรียนควรมีความสามารถดังนี้'</t>
+  </si>
+  <si>
+    <t>จับคู่กับคอลัมน์ 'การประเมินขั้นสำเร็จผล' เช่น การระบุข้อในใบงานหรือแบบทดสอบ</t>
+  </si>
+  <si>
+    <t>ต้องวัดผลให้ตรงตามพฤติกรรมที่ระบุในแต่ละวัตถุประสงค์เชิงพฤติกรรม โดยระบุหลักฐานการวัดผลในใบงานหรือแบบทดสอบ</t>
+  </si>
+  <si>
+    <t>ในแบบฟอร์มเริ่มต้นมีช่องกำหนดข้อ 1, 2, 3 และ 4 ไว้เป็นแนวทาง</t>
+  </si>
+  <si>
+    <t>ระบุทักษะหรือความรู้เดิมที่ผู้เรียนต้องมีก่อนเริ่มเรียนหัวข้อใหม่ เพื่อให้พร้อมต่อการรับบทเรียน</t>
+  </si>
+  <si>
+    <t>เป็นกิจกรรมหรือคำถามกระตุ้นความสนใจ เพื่อเชื่อมโยงประสบการณ์เดิมเข้าสู่เนื้อหาบทเรียนใหม่</t>
+  </si>
+  <si>
+    <t>เพื่อตรวจสอบความพร้อมของผู้เรียนและทบทวนความรู้เดิมก่อนต่อยอดไปยังเนื้อหาใหม่</t>
+  </si>
+  <si>
+    <t>มี 4 ขั้นตอนหลักตามแนวทาง MIAP ได้แก่ 1. ขั้นสนใจปัญหา (M) 2. ขั้นบอกกล่าว (I) 3. ขั้นพยายาม (A) และ 4. ขั้นสำเร็จผล (P)</t>
+  </si>
+  <si>
+    <t>ใช้ตัวย่อ '(I)' ซึ่งย่อมาจาก Information</t>
+  </si>
+  <si>
+    <t>ใช้ตัวย่อ '(A)' ซึ่งย่อมาจาก Application</t>
+  </si>
+  <si>
+    <t>ใช้ตัวย่อ '(P)' ซึ่งย่อมาจาก Progress</t>
+  </si>
+  <si>
+    <t>ตารางปฏิบัติการในแผนการสอนมีการแบ่งช่วงเวลาอย่างไร?</t>
+  </si>
+  <si>
+    <t>ตัวเลขสรุปโครงสร้างการสอนในแบบฟอร์มแสดงรหัสรูปแบบอะไร?</t>
+  </si>
+  <si>
+    <t>ในขั้นบอกกล่าว (I) มีเทคนิคการสอนย่อยอะไรให้เลือกติ๊กบ้าง?</t>
+  </si>
+  <si>
+    <t>หากครูต้องการอธิบายเนื้อหาหรือทฤษฎีในขั้นบอกกล่าว ควรเลือกช่องใด?</t>
+  </si>
+  <si>
+    <t>หากครูลงมือทำให้ดูเป็นตัวอย่างในขั้นบอกกล่าว ต้องระบุในช่องใด?</t>
+  </si>
+  <si>
+    <t>เทคนิค 'ชี้ทาง' ในขั้นบอกกล่าวคืออะไร?</t>
+  </si>
+  <si>
+    <t>เทคนิค 'สรุป' ในขั้นบอกกล่าวมีไว้เพื่ออะไร?</t>
+  </si>
+  <si>
+    <t>ในขั้นพยายาม (A) กำหนดรูปแบบกิจกรรมฝึกปฏิบัติไว้กี่รูปแบบ อะไรบ้าง?</t>
+  </si>
+  <si>
+    <t>การให้ผู้เรียนทำตามขั้นตอนที่ครูเพิ่งสาธิตไป จัดเป็นขั้นพยายามรูปแบบใด?</t>
+  </si>
+  <si>
+    <t>กิจกรรม 'แบบฝึกหัด' ในขั้นพยายามเน้นอะไร?</t>
+  </si>
+  <si>
+    <t>กิจกรรม 'แบบแก้ปัญหา' ในขั้นพยายาม เหมาะกับการเรียนการสอนแบบใด?</t>
+  </si>
+  <si>
+    <t>ตารางประเมินระดับกิจกรรมของผู้เรียนมีกี่ระดับ?</t>
+  </si>
+  <si>
+    <t>วัตถุประสงค์ของการบันทึก 'ระดับกิจกรรมผู้เรียน' ในแต่ละช่วงเวลาคืออะไร?</t>
+  </si>
+  <si>
+    <t>สิ่งสนับสนุนการเรียนการสอนในตารางมีรายการใดบ้าง?</t>
+  </si>
+  <si>
+    <t>หากใช้ PowerPoint หรือการฉายหน้าจอ ในแผนจัดอยู่ในหมวดสื่อใด?</t>
+  </si>
+  <si>
+    <t>หากมีการนำสาย LAN และคีมย้ำหัวของจริงมาใช้ จะตรงกับหมวดสื่อใด?</t>
+  </si>
+  <si>
+    <t>ถ้าครูใช้การเขียนสรุปหน้าห้อง จะจัดเป็นสื่อประเภทใดในแบบฟอร์ม?</t>
+  </si>
+  <si>
+    <t>ส่วน 'สิ่งที่แนบมาด้วย' ท้ายแผนการสอนประกอบด้วยเอกสารกี่ประเภท?</t>
+  </si>
+  <si>
+    <t>เอกสารแนบช่วยสนับสนุนการสอนของครูอย่างไร?</t>
+  </si>
+  <si>
+    <t>แบบร่างกระดาน (Board Plan) คืออะไร มีไว้เพื่อประโยชน์ใด?</t>
+  </si>
+  <si>
+    <t>มีการแบ่งช่องเวลาเป็นนาทีตั้งแต่ 1 ถึง 30 นาที และมีช่องสำหรับการบ้าน</t>
+  </si>
+  <si>
+    <t>ระบุโครงสร้างการสอนและรูปแบบการสอนที่เลือก เช่น รูปแบบ 1-2-3-4</t>
+  </si>
+  <si>
+    <t>มี 5 รูปแบบย่อย ได้แก่ บรรยาย, ถาม-ตอบ, สาธิต, ชี้ทาง และสรุป</t>
+  </si>
+  <si>
+    <t>เลือกรูปแบบ 'บรรยาย' หรือ 'ถาม-ตอบ' ตามลักษณะกิจกรรม</t>
+  </si>
+  <si>
+    <t>ระบุในช่อง 'สาธิต'</t>
+  </si>
+  <si>
+    <t>เป็นการแนะนำแนวทางหรือกระตุ้นให้ผู้เรียนค้นพบคำตอบด้วยตนเอง</t>
+  </si>
+  <si>
+    <t>ใช้สำหรับรวบยอดประเด็นสำคัญของเนื้อหาที่ได้บอกกล่าวไปให้ชัดเจนก่อนเริ่มขั้นพยายาม</t>
+  </si>
+  <si>
+    <t>มี 3 รูปแบบ ได้แก่ 1. แบบลอกเลียน 2. แบบฝึกหัด และ 3. แบบแก้ปัญหา</t>
+  </si>
+  <si>
+    <t>จัดเป็นกิจกรรม 'แบบลอกเลียน'</t>
+  </si>
+  <si>
+    <t>เน้นให้ผู้เรียนได้ฝึกฝนทบทวนและทำโจทย์เพื่อสร้างความเข้าใจที่มั่นคง</t>
+  </si>
+  <si>
+    <t>เหมาะกับโจทย์ที่มีความซับซ้อน หรือสถานการณ์จำลองที่ผู้เรียนต้องวิเคราะห์และประยุกต์ใช้ความรู้แก้ปัญหาด้วยตนเอง</t>
+  </si>
+  <si>
+    <t>แบ่งเป็น 3 ระดับ ได้แก่ ระดับสูง, ระดับปานกลาง และระดับต่ำ</t>
+  </si>
+  <si>
+    <t>เพื่อติดตามและตรวจสอบว่าผู้เรียนมีส่วนร่วม (Active Learning) มากน้อยเพียงใดตลอดแต่ละช่วงนาทีของการสอน</t>
+  </si>
+  <si>
+    <t>กระดาน, แผ่นภาพ, ใบเนื้อหา, ใบสั่งงาน, ใบทดสอบ, แผ่นใส/สไลด์, คอมพิวเตอร์, ของจริง/ตัวอย่าง และอุปกรณ์การทดลอง</t>
+  </si>
+  <si>
+    <t>จัดอยู่ในช่อง 'แผ่นใส / สไลด์' หรือ 'คอมพิวเตอร์'</t>
+  </si>
+  <si>
+    <t>ตรงกับหมวด 'ของจริง ตัวอย่าง' หรือ 'อุปกรณ์การทดลอง'</t>
+  </si>
+  <si>
+    <t>จัดอยู่ในช่อง 'กระดาน'</t>
+  </si>
+  <si>
+    <t>มี 6 ประเภท ได้แก่ แบบร่างกระดาน, ใบรายการถาม-ตอบ, ใบเนื้อหา, ใบงาน, ใบเฉลย และอื่น ๆ</t>
+  </si>
+  <si>
+    <t>ช่วยให้ครูเตรียมสื่อ เนื้อหา คำถาม-คำตอบ แบบฝึกหัด และการเขียนกระดานล่วงหน้าได้อย่างสมบูรณ์แบบและเป็นระบบ</t>
+  </si>
+  <si>
+    <t>เป็นการจำลองพื้นที่การเขียนกระดานล่วงหน้า เพื่อจัดสรรตำแหน่งหัวข้อ คำอธิบาย รูปภาพ และเฉลยให้เป็นระเบียบชัดเจน</t>
+  </si>
+  <si>
+    <t>ในแบบร่างกระดานมีการแบ่งแสดงเป็นกี่แผ่นตามตัวอย่าง?</t>
+  </si>
+  <si>
+    <t>ใบรายการถาม-ตอบ (Question &amp; Answer Sheet) ประกอบด้วยหัวข้ออะไรบ้าง?</t>
+  </si>
+  <si>
+    <t>ในใบรายการถาม-ตอบ มีการแยกการถามคำถามออกเป็นส่วนใดบ้าง?</t>
+  </si>
+  <si>
+    <t>ตัวอย่างคำถามที่ 1 ในการนำเข้าสู่บทเรียนคืออะไร?</t>
+  </si>
+  <si>
+    <t>ทำไมครูต้องเตรียมใบรายการถาม-ตอบไว้ล่วงหน้า?</t>
+  </si>
+  <si>
+    <t>ตัวอย่างมีการระบุเป็น แผ่นที่ 1/3, แผ่นที่ 2/3 และ แผ่นที่ 3/3 (รวมถึงเฉลยบนกระดาน)</t>
+  </si>
+  <si>
+    <t>ประกอบด้วย วัตถุประสงค์ (ข้อที่), รายการคำถาม และแนวคำตอบ</t>
+  </si>
+  <si>
+    <t>แยกเป็นส่วนคำถามใน 'การนำเข้าสู่บทเรียน' และคำถามที่ตรงตามแต่ละ 'วัตถุประสงค์' ของบทเรียน</t>
+  </si>
+  <si>
+    <t>คำถามคือ 'สวัสดีค่ะนักเรียน' และแนวคำตอบคือ 'สวัสดีครับ/ค่ะ'</t>
+  </si>
+  <si>
+    <t>เพื่อกำหนดทิศทางการตั้งคำถามกระตุ้นความคิด และเตรียมแนวคำตอบที่ถูกต้องไว้ตรวจสอบความเข้าใจของผู้เรียน</t>
+  </si>
+  <si>
+    <t>ใบเนื้อหาในเอกสารแนบระบุรายละเอียดหัวข้ออะไรไว้บ้าง?</t>
+  </si>
+  <si>
+    <t>ใบงานในแบบฟอร์มกำหนดโครงสร้างข้อมูลไว้อย่างไร?</t>
+  </si>
+  <si>
+    <t>ใบเฉลยในแผนการสอนคืออะไร?</t>
+  </si>
+  <si>
+    <t>ทำไมแผนการสอนจำเป็นต้องมีใบเฉลยแนบมาด้วย?</t>
+  </si>
+  <si>
+    <t>องค์ประกอบสำคัญที่ต้องมีในใบเฉลยมีอะไรบ้าง?</t>
+  </si>
+  <si>
+    <t>หากคำถามในใบงานเป็นคำถามปลายเปิด ใบเฉลยควรเขียนอย่างไร?</t>
+  </si>
+  <si>
+    <t>แหล่งข้อมูลหลักของบทเรียน (Primary Learning Resource)
+สรุปเนื้อหาที่ตรงตามจุดประสงค์เชิงพฤติกรรม โดยคัดกรองเฉพาะสาระสำคัญที่จำเป็น ไม่เยิ่นเย้อ ช่วยลดภาระการจดบันทึกของผู้เรียนและทำให้โฟกัสกับการทำความเข้าใจ
+เครื่องมือสนับสนุนการเรียนรู้ด้วยตนเอง (Self-Directed Learning)
+เปิดโอกาสให้ผู้เรียนศึกษาเนื้อหาตามจังหวะการเรียนรู้ของตนเอง (Self-paced) เหมาะกับการจัดการเรียนรู้แบบ Active Learning เช่น Flipped Classroom หรือการเรียนรู้แบบแก้ปัญหา (PBL)
+ฐานความรู้ก่อนลงมือปฏิบัติ (Theoretical Foundation)
+ในวิชาสายทักษะหรือปฏิบัติการ ใบเนื้อหาจะทำหน้าที่ปูพื้นฐานทฤษฎี คำศัพท์เฉพาะ ขั้นตอนการทำงาน และข้อควรระวัง ก่อนที่ผู้เรียนจะไปทำใบงาน (Worksheet) หรือใบปฏิบัติงาน (Job Sheet)
+สื่ออ้างอิงมาตรฐาน (Standardized Reference)
+ช่วยให้ผู้เรียนทุกคนได้รับชุดข้อมูลและมาตรฐานความรู้เดียวกัน แม้จะขาดเรียนหรือต้องการทบทวนย้อนหลัง</t>
+  </si>
+  <si>
+    <t>มีช่องระบุวิชา, ชั้น, เวลาทำ, ชื่อ-นามสกุล, รหัสประจำตัว, คำชี้แจง และรายการโจทย์ข้อคำถาม</t>
+  </si>
+  <si>
+    <t>เอกสารหรือสื่อประกอบการสอนสำหรับผู้สอน ที่ระบุคำตอบที่ถูกต้อง แสดงขั้นตอนวิธีคิด แนวทางการตอบ และเกณฑ์การให้คะแนนของใบงาน แบบฝึกหัด หรือแบบทดสอบ</t>
+  </si>
+  <si>
+    <t>เพื่อให้แผนการสอนมีความสมบูรณ์ตามมาตรฐานวิชาชีพครู ช่วยให้การประเมินผลมีความเที่ยงตรง และรองรับกรณีที่มีผู้สอนท่านอื่นนำแผนไปสอนแทนได้ทันทีโดยไม่ติดขัด</t>
+  </si>
+  <si>
+    <t>1. ส่วนหัว (ชื่อวิชา รหัสวิชา หน่วยการเรียน และอ้างอิงใบงานที่เกี่ยวข้อง)
+2. ส่วนคำตอบ/แนวคิด/ผลลัพธ์ที่คาดหวัง
+3. เกณฑ์การให้คะแนนและการกระจายคะแนนย่อย</t>
+  </si>
+  <si>
+    <t>ควรระบุเป็น "แนวคำตอบ" (Expected Key Points) โดยแจกแจงประเด็นสำคัญที่ผู้เรียนต้องตอบให้ครบ พร้อมเกณฑ์น้ำหนักคะแนนตามความลึกซึ้งของคำตอบ</t>
   </si>
 </sst>
 </file>
@@ -3514,7 +3830,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3524,6 +3840,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3827,12 +4146,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C952"/>
+  <dimension ref="A1:C1001"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="75" customWidth="1"/>
+    <col min="2" max="2" width="71.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="116.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -14307,6 +14626,594 @@
         <v>1077</v>
       </c>
     </row>
+    <row r="953" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A953">
+        <f>SUM(A952+1)</f>
+        <v>1001</v>
+      </c>
+      <c r="B953" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C953" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="954" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A954">
+        <f t="shared" ref="A954:A1001" si="0">SUM(A953+1)</f>
+        <v>1002</v>
+      </c>
+      <c r="B954" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C954" t="s">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="955" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A955">
+        <f t="shared" si="0"/>
+        <v>1003</v>
+      </c>
+      <c r="B955" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C955" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="956" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A956">
+        <f t="shared" si="0"/>
+        <v>1004</v>
+      </c>
+      <c r="B956" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C956" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="957" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A957">
+        <f t="shared" si="0"/>
+        <v>1005</v>
+      </c>
+      <c r="B957" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C957" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="958" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A958">
+        <f t="shared" si="0"/>
+        <v>1006</v>
+      </c>
+      <c r="B958" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C958" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="959" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A959">
+        <f t="shared" si="0"/>
+        <v>1007</v>
+      </c>
+      <c r="B959" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C959" t="s">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="960" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A960">
+        <f t="shared" si="0"/>
+        <v>1008</v>
+      </c>
+      <c r="B960" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C960" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="961" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A961">
+        <f t="shared" si="0"/>
+        <v>1009</v>
+      </c>
+      <c r="B961" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C961" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="962" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A962">
+        <f t="shared" si="0"/>
+        <v>1010</v>
+      </c>
+      <c r="B962" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C962" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="963" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A963">
+        <f t="shared" si="0"/>
+        <v>1011</v>
+      </c>
+      <c r="B963" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C963" t="s">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="964" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A964">
+        <f t="shared" si="0"/>
+        <v>1012</v>
+      </c>
+      <c r="B964" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C964" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="965" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A965">
+        <f t="shared" si="0"/>
+        <v>1013</v>
+      </c>
+      <c r="B965" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C965" t="s">
+        <v>1114</v>
+      </c>
+    </row>
+    <row r="966" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A966">
+        <f t="shared" si="0"/>
+        <v>1014</v>
+      </c>
+      <c r="B966" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C966" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="967" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A967">
+        <f t="shared" si="0"/>
+        <v>1015</v>
+      </c>
+      <c r="B967" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C967" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="968" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A968">
+        <f t="shared" si="0"/>
+        <v>1016</v>
+      </c>
+      <c r="B968" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C968" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="969" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A969">
+        <f t="shared" si="0"/>
+        <v>1017</v>
+      </c>
+      <c r="B969" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C969" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="970" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A970">
+        <f t="shared" si="0"/>
+        <v>1018</v>
+      </c>
+      <c r="B970" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C970" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="971" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A971">
+        <f t="shared" si="0"/>
+        <v>1019</v>
+      </c>
+      <c r="B971" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C971" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="972" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A972">
+        <f t="shared" si="0"/>
+        <v>1020</v>
+      </c>
+      <c r="B972" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C972" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="973" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A973">
+        <f t="shared" si="0"/>
+        <v>1021</v>
+      </c>
+      <c r="B973" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C973" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="974" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A974">
+        <f t="shared" si="0"/>
+        <v>1022</v>
+      </c>
+      <c r="B974" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C974" t="s">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="975" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A975">
+        <f t="shared" si="0"/>
+        <v>1023</v>
+      </c>
+      <c r="B975" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C975" t="s">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="976" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A976">
+        <f t="shared" si="0"/>
+        <v>1024</v>
+      </c>
+      <c r="B976" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C976" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="977" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A977">
+        <f t="shared" si="0"/>
+        <v>1025</v>
+      </c>
+      <c r="B977" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C977" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="978" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A978">
+        <f t="shared" si="0"/>
+        <v>1026</v>
+      </c>
+      <c r="B978" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C978" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="979" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A979">
+        <f t="shared" si="0"/>
+        <v>1027</v>
+      </c>
+      <c r="B979" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C979" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="980" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A980">
+        <f t="shared" si="0"/>
+        <v>1028</v>
+      </c>
+      <c r="B980" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C980" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="981" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A981">
+        <f t="shared" si="0"/>
+        <v>1029</v>
+      </c>
+      <c r="B981" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C981" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="982" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A982">
+        <f t="shared" si="0"/>
+        <v>1030</v>
+      </c>
+      <c r="B982" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C982" t="s">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="983" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A983">
+        <f t="shared" si="0"/>
+        <v>1031</v>
+      </c>
+      <c r="B983" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C983" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="984" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A984">
+        <f t="shared" si="0"/>
+        <v>1032</v>
+      </c>
+      <c r="B984" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C984" t="s">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="985" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A985">
+        <f t="shared" si="0"/>
+        <v>1033</v>
+      </c>
+      <c r="B985" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C985" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="986" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A986">
+        <f t="shared" si="0"/>
+        <v>1034</v>
+      </c>
+      <c r="B986" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C986" t="s">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="987" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A987">
+        <f t="shared" si="0"/>
+        <v>1035</v>
+      </c>
+      <c r="B987" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C987" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="988" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A988">
+        <f t="shared" si="0"/>
+        <v>1036</v>
+      </c>
+      <c r="B988" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C988" t="s">
+        <v>1157</v>
+      </c>
+    </row>
+    <row r="989" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A989">
+        <f t="shared" si="0"/>
+        <v>1037</v>
+      </c>
+      <c r="B989" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C989" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="990" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A990">
+        <f t="shared" si="0"/>
+        <v>1038</v>
+      </c>
+      <c r="B990" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C990" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="991" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A991">
+        <f t="shared" si="0"/>
+        <v>1039</v>
+      </c>
+      <c r="B991" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C991" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="992" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A992">
+        <f t="shared" si="0"/>
+        <v>1040</v>
+      </c>
+      <c r="B992" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C992" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="993" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A993">
+        <f t="shared" si="0"/>
+        <v>1041</v>
+      </c>
+      <c r="B993" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C993" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="994" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A994">
+        <f t="shared" si="0"/>
+        <v>1042</v>
+      </c>
+      <c r="B994" t="s">
+        <v>1163</v>
+      </c>
+      <c r="C994" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="995" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A995">
+        <f t="shared" si="0"/>
+        <v>1043</v>
+      </c>
+      <c r="B995" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C995" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="996" spans="1:3" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A996">
+        <f t="shared" si="0"/>
+        <v>1044</v>
+      </c>
+      <c r="B996" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C996" s="4" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="997" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A997">
+        <f t="shared" si="0"/>
+        <v>1045</v>
+      </c>
+      <c r="B997" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C997" t="s">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="998" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A998">
+        <f t="shared" si="0"/>
+        <v>1046</v>
+      </c>
+      <c r="B998" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C998" t="s">
+        <v>1178</v>
+      </c>
+    </row>
+    <row r="999" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A999">
+        <f t="shared" si="0"/>
+        <v>1047</v>
+      </c>
+      <c r="B999" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C999" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1000">
+        <f t="shared" si="0"/>
+        <v>1048</v>
+      </c>
+      <c r="B1000" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C1000" s="4" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1001">
+        <f t="shared" si="0"/>
+        <v>1049</v>
+      </c>
+      <c r="B1001" t="s">
+        <v>1175</v>
+      </c>
+      <c r="C1001" t="s">
+        <v>1181</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update QA dataset with new entries
</commit_message>
<xml_diff>
--- a/QA_Dataset_1000_Chatbot.xlsx
+++ b/QA_Dataset_1000_Chatbot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\doc-sheet-chatbot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B29FCA06-7BA6-4B7D-9B5A-D46AE0883C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2291720-DB9E-4C75-BE23-F9B7FDADB272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2003" uniqueCount="1182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2005" uniqueCount="1184">
   <si>
     <t>ลำดับข้อ</t>
   </si>
@@ -3744,6 +3744,12 @@
   </si>
   <si>
     <t>ควรระบุเป็น "แนวคำตอบ" (Expected Key Points) โดยแจกแจงประเด็นสำคัญที่ผู้เรียนต้องตอบให้ครบ พร้อมเกณฑ์น้ำหนักคะแนนตามความลึกซึ้งของคำตอบ</t>
+  </si>
+  <si>
+    <t>ใบเฉลยคืออะไร</t>
+  </si>
+  <si>
+    <t>ใบเฉลย (Answer Key / Solution Sheet) คือ เอกสารหรือสื่อที่รวบรวมคำตอบที่ถูกต้อง พร้อมแนวทางการตอบหรือวิธีทำของแบบทดสอบ แบบฝึกหัด หรือใบงาน โดยจัดทำขึ้นเพื่อใช้เป็นเกณฑ์มาตรฐานในการตรวจและประเมินผลการเรียนรู้</t>
   </si>
 </sst>
 </file>
@@ -4146,12 +4152,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1001"/>
+  <dimension ref="A1:C1002"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="71.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="116.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="193.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -15214,6 +15220,17 @@
         <v>1181</v>
       </c>
     </row>
+    <row r="1002" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1002">
+        <v>1050</v>
+      </c>
+      <c r="B1002" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C1002" t="s">
+        <v>1183</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>